<commit_message>
add 268-test suite covering pipeline invariants, models, and artifacts
</commit_message>
<xml_diff>
--- a/Corporate_Real_Estate_Management_Workbook.xlsx
+++ b/Corporate_Real_Estate_Management_Workbook.xlsx
@@ -2714,7 +2714,7 @@
         <v>58.77</v>
       </c>
       <c r="H5" s="25" t="n">
-        <v>78.89</v>
+        <v>87.31</v>
       </c>
       <c r="I5" s="25">
         <f>H5-G5</f>
@@ -2722,14 +2722,14 @@
       </c>
       <c r="J5" s="23" t="inlineStr">
         <is>
-          <t>Consistently active</t>
+          <t>Capacity-constrained</t>
         </is>
       </c>
       <c r="K5" s="15" t="n">
-        <v>3988</v>
+        <v>314</v>
       </c>
       <c r="L5" s="25" t="n">
-        <v>794.42</v>
+        <v>62.55</v>
       </c>
     </row>
     <row r="6">
@@ -2762,7 +2762,7 @@
         <v>44.61</v>
       </c>
       <c r="H6" s="31" t="n">
-        <v>64.79000000000001</v>
+        <v>74.89</v>
       </c>
       <c r="I6" s="31">
         <f>H6-G6</f>
@@ -2774,10 +2774,10 @@
         </is>
       </c>
       <c r="K6" s="30" t="n">
-        <v>413</v>
+        <v>194</v>
       </c>
       <c r="L6" s="31" t="n">
-        <v>82.27</v>
+        <v>38.65</v>
       </c>
     </row>
     <row r="7">
@@ -2810,7 +2810,7 @@
         <v>72.92</v>
       </c>
       <c r="H7" s="25" t="n">
-        <v>84.54000000000001</v>
+        <v>89.92</v>
       </c>
       <c r="I7" s="25">
         <f>H7-G7</f>
@@ -2822,10 +2822,10 @@
         </is>
       </c>
       <c r="K7" s="15" t="n">
-        <v>5505</v>
+        <v>366</v>
       </c>
       <c r="L7" s="25" t="n">
-        <v>1096.61</v>
+        <v>72.91</v>
       </c>
     </row>
     <row r="8">
@@ -2858,7 +2858,7 @@
         <v>65.88</v>
       </c>
       <c r="H8" s="31" t="n">
-        <v>83.3</v>
+        <v>89.81999999999999</v>
       </c>
       <c r="I8" s="31">
         <f>H8-G8</f>
@@ -2870,10 +2870,10 @@
         </is>
       </c>
       <c r="K8" s="30" t="n">
-        <v>7108</v>
+        <v>354</v>
       </c>
       <c r="L8" s="31" t="n">
-        <v>1415.94</v>
+        <v>70.52</v>
       </c>
     </row>
     <row r="9">
@@ -2906,7 +2906,7 @@
         <v>38.52</v>
       </c>
       <c r="H9" s="25" t="n">
-        <v>48.17</v>
+        <v>58.29</v>
       </c>
       <c r="I9" s="25">
         <f>H9-G9</f>
@@ -2954,7 +2954,7 @@
         <v>74.95999999999999</v>
       </c>
       <c r="H10" s="31" t="n">
-        <v>88.73999999999999</v>
+        <v>93.87</v>
       </c>
       <c r="I10" s="31">
         <f>H10-G10</f>
@@ -2966,10 +2966,10 @@
         </is>
       </c>
       <c r="K10" s="30" t="n">
-        <v>9513</v>
+        <v>404</v>
       </c>
       <c r="L10" s="31" t="n">
-        <v>1895.02</v>
+        <v>80.48</v>
       </c>
     </row>
     <row r="11">
@@ -3002,7 +3002,7 @@
         <v>69.89</v>
       </c>
       <c r="H11" s="25" t="n">
-        <v>85.26000000000001</v>
+        <v>90.55</v>
       </c>
       <c r="I11" s="25">
         <f>H11-G11</f>
@@ -3014,10 +3014,10 @@
         </is>
       </c>
       <c r="K11" s="15" t="n">
-        <v>5574</v>
+        <v>378</v>
       </c>
       <c r="L11" s="25" t="n">
-        <v>1110.36</v>
+        <v>75.3</v>
       </c>
     </row>
     <row r="12">
@@ -3050,7 +3050,7 @@
         <v>49.61</v>
       </c>
       <c r="H12" s="31" t="n">
-        <v>62.05</v>
+        <v>71.89</v>
       </c>
       <c r="I12" s="31">
         <f>H12-G12</f>
@@ -3062,10 +3062,10 @@
         </is>
       </c>
       <c r="K12" s="30" t="n">
-        <v>152</v>
+        <v>96</v>
       </c>
       <c r="L12" s="31" t="n">
-        <v>30.28</v>
+        <v>19.12</v>
       </c>
     </row>
     <row r="13">
@@ -3098,7 +3098,7 @@
         <v>62.8</v>
       </c>
       <c r="H13" s="25" t="n">
-        <v>80.59999999999999</v>
+        <v>88.29000000000001</v>
       </c>
       <c r="I13" s="25">
         <f>H13-G13</f>
@@ -3110,10 +3110,10 @@
         </is>
       </c>
       <c r="K13" s="15" t="n">
-        <v>4972</v>
+        <v>314</v>
       </c>
       <c r="L13" s="25" t="n">
-        <v>990.4400000000001</v>
+        <v>62.55</v>
       </c>
     </row>
     <row r="14">
@@ -3146,7 +3146,7 @@
         <v>42.59</v>
       </c>
       <c r="H14" s="31" t="n">
-        <v>52.06</v>
+        <v>61.39</v>
       </c>
       <c r="I14" s="31">
         <f>H14-G14</f>
@@ -3194,7 +3194,7 @@
         <v>70.91</v>
       </c>
       <c r="H15" s="25" t="n">
-        <v>86.56999999999999</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="I15" s="25">
         <f>H15-G15</f>
@@ -3206,10 +3206,10 @@
         </is>
       </c>
       <c r="K15" s="15" t="n">
-        <v>6769</v>
+        <v>396</v>
       </c>
       <c r="L15" s="25" t="n">
-        <v>1348.41</v>
+        <v>78.88</v>
       </c>
     </row>
     <row r="16">
@@ -3242,7 +3242,7 @@
         <v>53.73</v>
       </c>
       <c r="H16" s="31" t="n">
-        <v>75.03</v>
+        <v>84.12</v>
       </c>
       <c r="I16" s="31">
         <f>H16-G16</f>
@@ -3250,14 +3250,14 @@
       </c>
       <c r="J16" s="27" t="inlineStr">
         <is>
-          <t>Underutilized</t>
+          <t>Peak-sensitive</t>
         </is>
       </c>
       <c r="K16" s="30" t="n">
-        <v>1801</v>
+        <v>297</v>
       </c>
       <c r="L16" s="31" t="n">
-        <v>358.76</v>
+        <v>59.16</v>
       </c>
     </row>
     <row r="17">
@@ -3290,7 +3290,7 @@
         <v>63.81</v>
       </c>
       <c r="H17" s="25" t="n">
-        <v>83.86</v>
+        <v>90.18000000000001</v>
       </c>
       <c r="I17" s="25">
         <f>H17-G17</f>
@@ -3302,10 +3302,10 @@
         </is>
       </c>
       <c r="K17" s="15" t="n">
-        <v>5354</v>
+        <v>353</v>
       </c>
       <c r="L17" s="25" t="n">
-        <v>1066.53</v>
+        <v>70.31999999999999</v>
       </c>
     </row>
     <row r="18">
@@ -3338,7 +3338,7 @@
         <v>46.69</v>
       </c>
       <c r="H18" s="31" t="n">
-        <v>57.93</v>
+        <v>67.47</v>
       </c>
       <c r="I18" s="31">
         <f>H18-G18</f>
@@ -3350,10 +3350,10 @@
         </is>
       </c>
       <c r="K18" s="30" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="L18" s="31" t="n">
-        <v>4.18</v>
+        <v>3.39</v>
       </c>
     </row>
     <row r="19">
@@ -3386,7 +3386,7 @@
         <v>71.92</v>
       </c>
       <c r="H19" s="25" t="n">
-        <v>87.38</v>
+        <v>91.68000000000001</v>
       </c>
       <c r="I19" s="25">
         <f>H19-G19</f>
@@ -3398,10 +3398,10 @@
         </is>
       </c>
       <c r="K19" s="15" t="n">
-        <v>4010</v>
+        <v>393</v>
       </c>
       <c r="L19" s="25" t="n">
-        <v>798.8</v>
+        <v>78.29000000000001</v>
       </c>
     </row>
     <row r="20">
@@ -3434,7 +3434,7 @@
         <v>59.9</v>
       </c>
       <c r="H20" s="31" t="n">
-        <v>76.33</v>
+        <v>84.45999999999999</v>
       </c>
       <c r="I20" s="31">
         <f>H20-G20</f>
@@ -3442,14 +3442,14 @@
       </c>
       <c r="J20" s="27" t="inlineStr">
         <is>
-          <t>Consistently active</t>
+          <t>Capacity-constrained</t>
         </is>
       </c>
       <c r="K20" s="30" t="n">
-        <v>1915</v>
+        <v>298</v>
       </c>
       <c r="L20" s="31" t="n">
-        <v>381.47</v>
+        <v>59.36</v>
       </c>
     </row>
     <row r="21">
@@ -3482,7 +3482,7 @@
         <v>55.76</v>
       </c>
       <c r="H21" s="25" t="n">
-        <v>74.02</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="I21" s="25">
         <f>H21-G21</f>
@@ -3490,14 +3490,14 @@
       </c>
       <c r="J21" s="23" t="inlineStr">
         <is>
-          <t>Consistently active</t>
+          <t>Capacity-constrained</t>
         </is>
       </c>
       <c r="K21" s="15" t="n">
-        <v>1632</v>
+        <v>293</v>
       </c>
       <c r="L21" s="25" t="n">
-        <v>325.1</v>
+        <v>58.37</v>
       </c>
     </row>
     <row r="22">
@@ -3530,7 +3530,7 @@
         <v>48.59</v>
       </c>
       <c r="H22" s="31" t="n">
-        <v>61.3</v>
+        <v>71.12</v>
       </c>
       <c r="I22" s="31">
         <f>H22-G22</f>
@@ -3542,10 +3542,10 @@
         </is>
       </c>
       <c r="K22" s="30" t="n">
-        <v>124</v>
+        <v>92</v>
       </c>
       <c r="L22" s="31" t="n">
-        <v>24.7</v>
+        <v>18.33</v>
       </c>
     </row>
     <row r="23">
@@ -3578,7 +3578,7 @@
         <v>52.81</v>
       </c>
       <c r="H23" s="25" t="n">
-        <v>74.92</v>
+        <v>82.8</v>
       </c>
       <c r="I23" s="25">
         <f>H23-G23</f>
@@ -3586,14 +3586,14 @@
       </c>
       <c r="J23" s="23" t="inlineStr">
         <is>
-          <t>Underutilized</t>
+          <t>Peak-sensitive</t>
         </is>
       </c>
       <c r="K23" s="15" t="n">
-        <v>1135</v>
+        <v>285</v>
       </c>
       <c r="L23" s="25" t="n">
-        <v>226.1</v>
+        <v>56.77</v>
       </c>
     </row>
     <row r="24">
@@ -3626,7 +3626,7 @@
         <v>41.51</v>
       </c>
       <c r="H24" s="31" t="n">
-        <v>50.73</v>
+        <v>59.3</v>
       </c>
       <c r="I24" s="31">
         <f>H24-G24</f>
@@ -3674,7 +3674,7 @@
         <v>60.82</v>
       </c>
       <c r="H25" s="25" t="n">
-        <v>81.08</v>
+        <v>87.66</v>
       </c>
       <c r="I25" s="25">
         <f>H25-G25</f>
@@ -3686,10 +3686,10 @@
         </is>
       </c>
       <c r="K25" s="15" t="n">
-        <v>2538</v>
+        <v>317</v>
       </c>
       <c r="L25" s="25" t="n">
-        <v>505.58</v>
+        <v>63.15</v>
       </c>
     </row>
     <row r="26">
@@ -3722,7 +3722,7 @@
         <v>54.83</v>
       </c>
       <c r="H26" s="31" t="n">
-        <v>68.45999999999999</v>
+        <v>78.06</v>
       </c>
       <c r="I26" s="31">
         <f>H26-G26</f>
@@ -3734,10 +3734,10 @@
         </is>
       </c>
       <c r="K26" s="30" t="n">
-        <v>1139</v>
+        <v>271</v>
       </c>
       <c r="L26" s="31" t="n">
-        <v>226.89</v>
+        <v>53.98</v>
       </c>
     </row>
     <row r="27">
@@ -3770,7 +3770,7 @@
         <v>64.84999999999999</v>
       </c>
       <c r="H27" s="25" t="n">
-        <v>84.20999999999999</v>
+        <v>89.83</v>
       </c>
       <c r="I27" s="25">
         <f>H27-G27</f>
@@ -3782,10 +3782,10 @@
         </is>
       </c>
       <c r="K27" s="15" t="n">
-        <v>3643</v>
+        <v>352</v>
       </c>
       <c r="L27" s="25" t="n">
-        <v>725.7</v>
+        <v>70.12</v>
       </c>
     </row>
     <row r="28">
@@ -3818,7 +3818,7 @@
         <v>56.78</v>
       </c>
       <c r="H28" s="31" t="n">
-        <v>73.18000000000001</v>
+        <v>81.81</v>
       </c>
       <c r="I28" s="31">
         <f>H28-G28</f>
@@ -3826,14 +3826,14 @@
       </c>
       <c r="J28" s="27" t="inlineStr">
         <is>
-          <t>Consistently active</t>
+          <t>Capacity-constrained</t>
         </is>
       </c>
       <c r="K28" s="30" t="n">
-        <v>1439</v>
+        <v>281</v>
       </c>
       <c r="L28" s="31" t="n">
-        <v>286.65</v>
+        <v>55.98</v>
       </c>
     </row>
     <row r="29">
@@ -3866,7 +3866,7 @@
         <v>47.59</v>
       </c>
       <c r="H29" s="25" t="n">
-        <v>65.65000000000001</v>
+        <v>73.77</v>
       </c>
       <c r="I29" s="25">
         <f>H29-G29</f>
@@ -3878,10 +3878,10 @@
         </is>
       </c>
       <c r="K29" s="15" t="n">
-        <v>246</v>
+        <v>153</v>
       </c>
       <c r="L29" s="25" t="n">
-        <v>49</v>
+        <v>30.48</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
add portfolio metadata badges and executive report briefing to README
</commit_message>
<xml_diff>
--- a/Corporate_Real_Estate_Management_Workbook.xlsx
+++ b/Corporate_Real_Estate_Management_Workbook.xlsx
@@ -8613,7 +8613,7 @@
     <col width="42" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
@@ -8765,7 +8765,7 @@
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>Lead Analyst</t>
+          <t>Hriday Singh Sobti</t>
         </is>
       </c>
       <c r="E11" s="23" t="inlineStr">
@@ -8798,7 +8798,7 @@
       </c>
       <c r="K11" s="14" t="inlineStr">
         <is>
-          <t>Verified Python 3.14 openpyxl duckdb reportlab pptx</t>
+          <t>Configured Python 3.14 environment and verified DuckDB openpyxl reportlab and pytest toolchains</t>
         </is>
       </c>
       <c r="L11" s="23" t="inlineStr">
@@ -8825,7 +8825,7 @@
       </c>
       <c r="D12" s="28" t="inlineStr">
         <is>
-          <t>Lead Analyst</t>
+          <t>Hriday Singh Sobti</t>
         </is>
       </c>
       <c r="E12" s="27" t="inlineStr">
@@ -8858,7 +8858,7 @@
       </c>
       <c r="K12" s="28" t="inlineStr">
         <is>
-          <t>Authored docs/research_notes.md covering 20 CRE topics</t>
+          <t>Synthesized BOMA Z65.1 loss factor formulas and CBRE APAC office rental benchmarks into notes</t>
         </is>
       </c>
       <c r="L12" s="27" t="inlineStr">
@@ -8885,7 +8885,7 @@
       </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
-          <t>Lead Analyst</t>
+          <t>Hriday Singh Sobti</t>
         </is>
       </c>
       <c r="E13" s="23" t="inlineStr">
@@ -8918,7 +8918,7 @@
       </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
-          <t>Authored data and metric dictionaries with strict constraints</t>
+          <t>Drafted star schema dimensional entities and metric dictionary with strict constraints</t>
         </is>
       </c>
       <c r="L13" s="23" t="inlineStr">
@@ -8945,7 +8945,7 @@
       </c>
       <c r="D14" s="28" t="inlineStr">
         <is>
-          <t>Lead Analyst</t>
+          <t>Hriday Singh Sobti</t>
         </is>
       </c>
       <c r="E14" s="27" t="inlineStr">
@@ -8978,7 +8978,7 @@
       </c>
       <c r="K14" s="28" t="inlineStr">
         <is>
-          <t>Generated 25 properties 112 floors 809 spaces and 282k fact rows</t>
+          <t>Built NumPy/Pandas generator with Beta distributions for 25 properties and 282k fact rows</t>
         </is>
       </c>
       <c r="L14" s="27" t="inlineStr">
@@ -9005,7 +9005,7 @@
       </c>
       <c r="D15" s="14" t="inlineStr">
         <is>
-          <t>Data Quality Engineer</t>
+          <t>Hriday Singh Sobti</t>
         </is>
       </c>
       <c r="E15" s="23" t="inlineStr">
@@ -9038,7 +9038,7 @@
       </c>
       <c r="K15" s="14" t="inlineStr">
         <is>
-          <t>Injected 44 realistic defects across 6 dimensions into raw layer</t>
+          <t>Injected 44 operational data defects across 6 dimensions to exercise cleaning pipeline</t>
         </is>
       </c>
       <c r="L15" s="23" t="inlineStr">
@@ -9065,7 +9065,7 @@
       </c>
       <c r="D16" s="28" t="inlineStr">
         <is>
-          <t>Data Quality Engineer</t>
+          <t>Hriday Singh Sobti</t>
         </is>
       </c>
       <c r="E16" s="27" t="inlineStr">
@@ -9098,7 +9098,7 @@
       </c>
       <c r="K16" s="28" t="inlineStr">
         <is>
-          <t>Codified rules DQ001 to DQ012 with 99.98% pass rate verification</t>
+          <t>Wrote automated DQ rules engine in Python (DQ001-DQ012) and verified 99.98% pass rate</t>
         </is>
       </c>
       <c r="L16" s="27" t="inlineStr">
@@ -9125,7 +9125,7 @@
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
-          <t>Data Quality Engineer</t>
+          <t>Hriday Singh Sobti</t>
         </is>
       </c>
       <c r="E17" s="23" t="inlineStr">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="K17" s="14" t="inlineStr">
         <is>
-          <t>Standardized geocoding and resolved all 44 manifest issues</t>
+          <t>Implemented cleaning pipeline for date inversion capacity bounding and area loss reconciliations</t>
         </is>
       </c>
       <c r="L17" s="23" t="inlineStr">
@@ -9185,7 +9185,7 @@
       </c>
       <c r="D18" s="28" t="inlineStr">
         <is>
-          <t>SQL Developer</t>
+          <t>Hriday Singh Sobti</t>
         </is>
       </c>
       <c r="E18" s="27" t="inlineStr">
@@ -9218,7 +9218,7 @@
       </c>
       <c r="K18" s="28" t="inlineStr">
         <is>
-          <t>Loaded 12 tables into relational DB with 0 FK violations</t>
+          <t>Loaded clean tables into DuckDB relational schema with primary keys checks and foreign keys</t>
         </is>
       </c>
       <c r="L18" s="27" t="inlineStr">
@@ -9245,7 +9245,7 @@
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
-          <t>SQL Developer</t>
+          <t>Hriday Singh Sobti</t>
         </is>
       </c>
       <c r="E19" s="23" t="inlineStr">
@@ -9278,7 +9278,7 @@
       </c>
       <c r="K19" s="14" t="inlineStr">
         <is>
-          <t>Implemented 16 business queries and 7 analytical reporting views</t>
+          <t>Wrote 16 analytical SQL queries with CTEs window functions and created 7 reporting views</t>
         </is>
       </c>
       <c r="L19" s="23" t="inlineStr">
@@ -9305,7 +9305,7 @@
       </c>
       <c r="D20" s="28" t="inlineStr">
         <is>
-          <t>BI Analyst</t>
+          <t>Hriday Singh Sobti</t>
         </is>
       </c>
       <c r="E20" s="27" t="inlineStr">
@@ -9338,7 +9338,7 @@
       </c>
       <c r="K20" s="28" t="inlineStr">
         <is>
-          <t>Generated 5 publication charts for weekday matrix cost and PAI</t>
+          <t>Generated Matplotlib/Seaborn diagnostic plots for weekday profiles and pressure matrix</t>
         </is>
       </c>
       <c r="L20" s="27" t="inlineStr">
@@ -9365,7 +9365,7 @@
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>BI Analyst</t>
+          <t>Hriday Singh Sobti</t>
         </is>
       </c>
       <c r="E21" s="23" t="inlineStr">
@@ -9398,7 +9398,7 @@
       </c>
       <c r="K21" s="14" t="inlineStr">
         <is>
-          <t>Validated 5-factor PAI with Spearman rho &gt; 0.97 across 4 schemes</t>
+          <t>Implemented Portfolio Attention Index (PAI) with Spearman rank correlation sensitivity checks</t>
         </is>
       </c>
       <c r="L21" s="23" t="inlineStr">
@@ -9425,7 +9425,7 @@
       </c>
       <c r="D22" s="28" t="inlineStr">
         <is>
-          <t>Lead Analyst</t>
+          <t>Hriday Singh Sobti</t>
         </is>
       </c>
       <c r="E22" s="27" t="inlineStr">
@@ -9458,7 +9458,7 @@
       </c>
       <c r="K22" s="28" t="inlineStr">
         <is>
-          <t>Modeled 10% 15% and 20% seat surrender scenarios with cost elasticity</t>
+          <t>Built 3-tier space consolidation model with 60% variable cost elasticity assumption</t>
         </is>
       </c>
       <c r="L22" s="27" t="inlineStr">
@@ -9485,7 +9485,7 @@
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
-          <t>BI Developer</t>
+          <t>Hriday Singh Sobti</t>
         </is>
       </c>
       <c r="E23" s="23" t="inlineStr">
@@ -9518,7 +9518,7 @@
       </c>
       <c r="K23" s="14" t="inlineStr">
         <is>
-          <t>Created Model.bim theme.json and 31 explicit DAX measures</t>
+          <t>Authored Model.bim Tabular schema 31 explicit DAX measures and corporate theme JSON</t>
         </is>
       </c>
       <c r="L23" s="23" t="inlineStr">
@@ -9545,7 +9545,7 @@
       </c>
       <c r="D24" s="28" t="inlineStr">
         <is>
-          <t>BI Developer</t>
+          <t>Hriday Singh Sobti</t>
         </is>
       </c>
       <c r="E24" s="27" t="inlineStr">
@@ -9578,7 +9578,7 @@
       </c>
       <c r="K24" s="28" t="inlineStr">
         <is>
-          <t>Specified executive layout pressure matrix and drill-through views</t>
+          <t>Drafted 6 core report page layout specifications and Property Detail drill-through layout</t>
         </is>
       </c>
       <c r="L24" s="27" t="inlineStr">
@@ -9605,7 +9605,7 @@
       </c>
       <c r="D25" s="14" t="inlineStr">
         <is>
-          <t>Front-End / BI Developer</t>
+          <t>Hriday Singh Sobti</t>
         </is>
       </c>
       <c r="E25" s="23" t="inlineStr">
@@ -9638,7 +9638,7 @@
       </c>
       <c r="K25" s="14" t="inlineStr">
         <is>
-          <t>Deployed zero-dependency interactive dashboard with working slicers</t>
+          <t>Built zero-dependency web dashboard preview with instant synchronous data and active slicers</t>
         </is>
       </c>
       <c r="L25" s="23" t="inlineStr">
@@ -9665,7 +9665,7 @@
       </c>
       <c r="D26" s="28" t="inlineStr">
         <is>
-          <t>Financial Analyst</t>
+          <t>Hriday Singh Sobti</t>
         </is>
       </c>
       <c r="E26" s="27" t="inlineStr">
@@ -9698,7 +9698,7 @@
       </c>
       <c r="K26" s="28" t="inlineStr">
         <is>
-          <t>Built 8-sheet workbook with live formulas formatting and freeze panes</t>
+          <t>Built 8-sheet Excel management workbook using openpyxl with 307 verified dynamic cell formulas</t>
         </is>
       </c>
       <c r="L26" s="27" t="inlineStr">
@@ -9725,7 +9725,7 @@
       </c>
       <c r="D27" s="14" t="inlineStr">
         <is>
-          <t>Report Designer</t>
+          <t>Hriday Singh Sobti</t>
         </is>
       </c>
       <c r="E27" s="23" t="inlineStr">
@@ -9758,7 +9758,7 @@
       </c>
       <c r="K27" s="14" t="inlineStr">
         <is>
-          <t>Typeset publication-grade PDF with embedded charts and evidence</t>
+          <t>Typeset 10-page management briefing PDF using ReportLab with dynamic NumberedCanvas page numbering</t>
         </is>
       </c>
       <c r="L27" s="23" t="inlineStr">
@@ -9785,7 +9785,7 @@
       </c>
       <c r="D28" s="28" t="inlineStr">
         <is>
-          <t>Presentation Specialist</t>
+          <t>Hriday Singh Sobti</t>
         </is>
       </c>
       <c r="E28" s="27" t="inlineStr">
@@ -9818,7 +9818,7 @@
       </c>
       <c r="K28" s="28" t="inlineStr">
         <is>
-          <t>Designed corporate PPTX deck with message headlines and callouts</t>
+          <t>Constructed 7-slide executive PowerPoint deck using python-pptx with 16:9 widescreen layout</t>
         </is>
       </c>
       <c r="L28" s="27" t="inlineStr">
@@ -9845,7 +9845,7 @@
       </c>
       <c r="D29" s="14" t="inlineStr">
         <is>
-          <t>QA Engineer</t>
+          <t>Hriday Singh Sobti</t>
         </is>
       </c>
       <c r="E29" s="23" t="inlineStr">
@@ -9878,7 +9878,7 @@
       </c>
       <c r="K29" s="14" t="inlineStr">
         <is>
-          <t>Implemented pytest suite verifying constraints and calculations</t>
+          <t>Wrote 268 automated pytest test cases covering schema DQ invariants and SQL parity</t>
         </is>
       </c>
       <c r="L29" s="23" t="inlineStr">
@@ -9905,7 +9905,7 @@
       </c>
       <c r="D30" s="28" t="inlineStr">
         <is>
-          <t>Lead Analyst</t>
+          <t>Hriday Singh Sobti</t>
         </is>
       </c>
       <c r="E30" s="27" t="inlineStr">
@@ -9938,7 +9938,7 @@
       </c>
       <c r="K30" s="28" t="inlineStr">
         <is>
-          <t>Reconciled totals across Python SQL Power BI and Excel</t>
+          <t>Audited cross-platform totals across Python SQL Power BI and Excel; confirmed 0.00% variance</t>
         </is>
       </c>
       <c r="L30" s="27" t="inlineStr">
@@ -9965,7 +9965,7 @@
       </c>
       <c r="D31" s="14" t="inlineStr">
         <is>
-          <t>Lead Designer</t>
+          <t>Hriday Singh Sobti</t>
         </is>
       </c>
       <c r="E31" s="23" t="inlineStr">
@@ -9998,7 +9998,7 @@
       </c>
       <c r="K31" s="14" t="inlineStr">
         <is>
-          <t>Rendered PDF and slides to images and verified visual bounds</t>
+          <t>Rendered PDF pages to 144 DPI PNGs via pypdfium2 to visually inspect typography and bounds</t>
         </is>
       </c>
       <c r="L31" s="23" t="inlineStr">
@@ -10020,12 +10020,12 @@
       </c>
       <c r="C32" s="28" t="inlineStr">
         <is>
-          <t>Perform humanization audit and finalize README portfolio</t>
+          <t>Perform editorial review and finalize README project documentation</t>
         </is>
       </c>
       <c r="D32" s="28" t="inlineStr">
         <is>
-          <t>Lead Analyst</t>
+          <t>Hriday Singh Sobti</t>
         </is>
       </c>
       <c r="E32" s="27" t="inlineStr">
@@ -10058,7 +10058,7 @@
       </c>
       <c r="K32" s="28" t="inlineStr">
         <is>
-          <t>Removed generic AI buzzwords and finalized GitHub portfolio structure</t>
+          <t>Conducted final review of repository documentation structure and operational terminology</t>
         </is>
       </c>
       <c r="L32" s="27" t="inlineStr">

</xml_diff>